<commit_message>
Updated docs in support of I-20 — Configuration Separation implementation.
</commit_message>
<xml_diff>
--- a/implementation/policy-assistant-inventory-list/policy-assist-apps-resource-inventory-sheet-v2.xlsx
+++ b/implementation/policy-assistant-inventory-list/policy-assist-apps-resource-inventory-sheet-v2.xlsx
@@ -8,20 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Steven\GitHub-Repositories\Repositories\azure-policy-assistant-rag-solution-docs\implementation\policy-assistant-inventory-list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{068B3792-2A18-492E-B77A-D29E2E29B2DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45FEA559-5577-4122-BAD1-A795EBF6B1A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Inventory By Platform" sheetId="1" r:id="rId1"/>
+    <sheet name="Inventory By Environment" sheetId="2" r:id="rId2"/>
+    <sheet name="Weights" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory By Platform'!$A$2:$G$42</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="271">
   <si>
     <t>Policy Assistant Client &amp; Orchestration Resource Inventory — Platform identifies where the resource lives, is configured, or is stored.</t>
   </si>
@@ -152,9 +156,6 @@
     <t>Azure AI Search Service</t>
   </si>
   <si>
-    <t>Azure AI Search</t>
-  </si>
-  <si>
     <t>Development search service used by the orchestration Function App.</t>
   </si>
   <si>
@@ -509,9 +510,6 @@
     <t>Development - Static Web App - Resource</t>
   </si>
   <si>
-    <t>Default Hostname</t>
-  </si>
-  <si>
     <t>polite-ground-0d2a97a1e.6.azurestaticapps.net</t>
   </si>
   <si>
@@ -519,6 +517,327 @@
   </si>
   <si>
     <t>Development Redirect URI</t>
+  </si>
+  <si>
+    <t>Default - Hostname</t>
+  </si>
+  <si>
+    <t>COSMOS_ENDPOINT</t>
+  </si>
+  <si>
+    <t>COSMOS_DATABASE_NAME</t>
+  </si>
+  <si>
+    <t>COSMOS_DATABASE</t>
+  </si>
+  <si>
+    <t>COSMOS_CONVERSATIONS_CONTAINER</t>
+  </si>
+  <si>
+    <t>COSMOS_MESSAGES_CONTAINER</t>
+  </si>
+  <si>
+    <t>AZURE_SEARCH_ENDPOINT</t>
+  </si>
+  <si>
+    <t>AZURE_SEARCH_INDEX_NAME</t>
+  </si>
+  <si>
+    <t>AZURE_SEARCH_CONTENT_FIELD</t>
+  </si>
+  <si>
+    <t>AZURE_SEARCH_VECTOR_FIELD</t>
+  </si>
+  <si>
+    <t>AZURE_SEARCH_SOURCE_FIELD</t>
+  </si>
+  <si>
+    <t>AZURE_OPENAI_ENDPOINT</t>
+  </si>
+  <si>
+    <t>AZURE_OPENAI_DEPLOYMENT</t>
+  </si>
+  <si>
+    <t>ENTRA_TENANT_ID</t>
+  </si>
+  <si>
+    <t>ENTRA_API_CLIENT_ID</t>
+  </si>
+  <si>
+    <t>OBO_TENANT_ID</t>
+  </si>
+  <si>
+    <t>OBO_CLIENT_ID</t>
+  </si>
+  <si>
+    <t>OBO_CLIENT_SECRET</t>
+  </si>
+  <si>
+    <t>POLICY_SYSTEM_PROMPT_VERSION</t>
+  </si>
+  <si>
+    <t>POLICY_SYSTEM_PROMPT_FILE</t>
+  </si>
+  <si>
+    <t>chunk</t>
+  </si>
+  <si>
+    <t>text_vector</t>
+  </si>
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>Foundry AI Search</t>
+  </si>
+  <si>
+    <t>Foundry - OpenAI</t>
+  </si>
+  <si>
+    <t>Entra ID</t>
+  </si>
+  <si>
+    <t>cfc6f96e-9d3c-4b29-b09d-44bab3055d31</t>
+  </si>
+  <si>
+    <t>On-Behalf-Of Token</t>
+  </si>
+  <si>
+    <t>&lt;ROTATE_AND_INSERT_NEW_SECRET_HERE&gt;</t>
+  </si>
+  <si>
+    <t>3.0</t>
+  </si>
+  <si>
+    <t>prompts/policy_assistant_system_v3.txt</t>
+  </si>
+  <si>
+    <t>LLM Policy System Prompt</t>
+  </si>
+  <si>
+    <t>function_app.py:27:    os.getenv("MAX_RAW_HISTORY_MESSAGES", "12")</t>
+  </si>
+  <si>
+    <t>function_app.py:31:    os.getenv("SUMMARY_TRIGGER_MESSAGE_COUNT", "20")</t>
+  </si>
+  <si>
+    <t>function_app.py:35:    os.getenv("MAX_CONVERSATION_CONTEXT_TOKENS", "12000")</t>
+  </si>
+  <si>
+    <t>function_app.py:39:    os.getenv("RESERVED_SEARCH_EVIDENCE_TOKENS", "3000")</t>
+  </si>
+  <si>
+    <t>function_app.py:43:    os.getenv("RESERVED_CURRENT_QUESTION_TOKENS", "750")</t>
+  </si>
+  <si>
+    <t>function_app.py:47:    os.getenv("RESERVED_RESPONSE_TOKENS", "2000")</t>
+  </si>
+  <si>
+    <t>function_app.py:55:    os.getenv("CONTEXT_OVERHEAD_SAFETY_TOKENS", "250")</t>
+  </si>
+  <si>
+    <t>function_app.py:62:    os.getenv("RECENT_RAW_HISTORY_TOKEN_BUDGET", "3000")</t>
+  </si>
+  <si>
+    <t>function_app.py:66:    os.getenv("SUMMARY_HISTORY_TOKEN_BUDGET", "1250")</t>
+  </si>
+  <si>
+    <t>function_app.py:70:    os.getenv("SUMMARY_MAX_TOKENS", "1200")</t>
+  </si>
+  <si>
+    <t>function_app.py:81:    os.getenv("MEMORY_LOOKBACK_DAYS", "180")</t>
+  </si>
+  <si>
+    <t>function_app.py:85:    os.getenv("MEMORY_CANDIDATE_LIMIT", "75")</t>
+  </si>
+  <si>
+    <t>function_app.py:89:    os.getenv("MEMORY_PREFILTER_LIMIT", "25")</t>
+  </si>
+  <si>
+    <t>function_app.py:93:    os.getenv("MEMORY_TOP_K", "10")</t>
+  </si>
+  <si>
+    <t>function_app.py:97:    os.getenv("MEMORY_MIN_RELEVANCE", "0.45")</t>
+  </si>
+  <si>
+    <t>function_app.py:101:    os.getenv("MEMORY_CONTEXT_TOKEN_BUDGET", "1000")</t>
+  </si>
+  <si>
+    <t>function_app.py:112:    os.getenv("I29_TEST_C_MIN_RELEVANCE", "1.01")</t>
+  </si>
+  <si>
+    <t>function_app.py:350:    os.getenv("MEMORY_EXTRACTION_MAX_MESSAGES", "12")</t>
+  </si>
+  <si>
+    <t>function_app.py:354:    os.getenv("MEMORY_EXTRACTION_MAX_OUTPUT_TOKENS", "1200")</t>
+  </si>
+  <si>
+    <t>function_app.py:360:    os.getenv("MEMORY_EXTRACTION_MAX_CHARS_PER_MESSAGE", "6000")</t>
+  </si>
+  <si>
+    <t>function_app.py:370:    os.getenv("LONG_TERM_MEMORY_MAX_ITEM_CHARS", "1000")</t>
+  </si>
+  <si>
+    <t>function_app.py:374:    os.getenv("LONG_TERM_MEMORY_MIN_CONFIDENCE", "0.75")</t>
+  </si>
+  <si>
+    <t>function_app.py:378:    os.getenv("LONG_TERM_MEMORY_MIN_IMPORTANCE", "0.50")</t>
+  </si>
+  <si>
+    <t>function_app.py:412:    os.getenv("LONG_TERM_MEMORY_ENABLED", "true")</t>
+  </si>
+  <si>
+    <t>function_app.py:428:    os.getenv("MEMORY_CANDIDATE_LOOKBACK_DAYS", "180")</t>
+  </si>
+  <si>
+    <t>function_app.py:432:    os.getenv("MEMORY_DEFAULT_RETENTION_DAYS", "180")</t>
+  </si>
+  <si>
+    <t>function_app.py:436:    os.getenv("MEMORY_MAX_CANDIDATES", "200")</t>
+  </si>
+  <si>
+    <t>function_app.py:440:    os.getenv("MEMORY_MAX_RETRIEVED_ITEMS", "10")</t>
+  </si>
+  <si>
+    <t>function_app.py:444:    os.getenv("MEMORY_RELEVANCE_THRESHOLD", "0.65")</t>
+  </si>
+  <si>
+    <t>function_app.py:448:    os.getenv("MEMORY_TOKEN_BUDGET", "1500")</t>
+  </si>
+  <si>
+    <t>function_app.py:457:    os.getenv("MEMORY_ALLOW_USER_PREFERENCES", "true")</t>
+  </si>
+  <si>
+    <t>function_app.py:464:    os.getenv("MEMORY_ALLOW_PROJECT_CONTEXT", "true")</t>
+  </si>
+  <si>
+    <t>function_app.py:471:    os.getenv("MEMORY_ALLOW_DURABLE_FACTS", "true")</t>
+  </si>
+  <si>
+    <t>function_app.py:483:    os.getenv("MEMORY_ALLOW_POLICY_CONTENT", "false")</t>
+  </si>
+  <si>
+    <t>function_app.py:490:    os.getenv("MEMORY_ALLOW_AUTHORIZATION_DATA", "false")</t>
+  </si>
+  <si>
+    <t>function_app.py:497:    os.getenv("MEMORY_ALLOW_SECRETS", "false")</t>
+  </si>
+  <si>
+    <t>function_app.py:531:    os.getenv("MEMORY_AUDIT_ENABLED", "true")</t>
+  </si>
+  <si>
+    <t>function_app.py:629:    os.getenv("MEMORY_RETRIEVAL_MAX_ITEMS", "8")</t>
+  </si>
+  <si>
+    <t>function_app.py:633:    os.getenv("MEMORY_RETRIEVAL_MAX_CHARS", "6000")</t>
+  </si>
+  <si>
+    <t>function_app.py:642:    os.getenv("MEMORY_DEV_VALIDATION_ENABLED", "false")</t>
+  </si>
+  <si>
+    <t>function_app.py:1106:    os.getenv("I28_COMPLETION_REPORT_ENABLED", "true")</t>
+  </si>
+  <si>
+    <t>function_app.py:1113:    os.getenv(</t>
+  </si>
+  <si>
+    <t>function_app.py:1132:    os.getenv("FORCE_SUMMARY_FAILURE_TEST", "false").strip().lower()</t>
+  </si>
+  <si>
+    <t>function_app.py:1142:OBO_TENANT_ID = os.environ["OBO_TENANT_ID"]</t>
+  </si>
+  <si>
+    <t>function_app.py:1143:OBO_CLIENT_ID = os.environ["OBO_CLIENT_ID"]</t>
+  </si>
+  <si>
+    <t>function_app.py:1144:OBO_CLIENT_SECRET = os.environ["OBO_CLIENT_SECRET"]</t>
+  </si>
+  <si>
+    <t>function_app.py:1163:SEARCH_ENDPOINT = os.environ["AZURE_SEARCH_ENDPOINT"]</t>
+  </si>
+  <si>
+    <t>function_app.py:1164:SEARCH_INDEX_NAME = os.environ["AZURE_SEARCH_INDEX_NAME"]</t>
+  </si>
+  <si>
+    <t>function_app.py:1166:CONTENT_FIELD = os.environ["AZURE_SEARCH_CONTENT_FIELD"]</t>
+  </si>
+  <si>
+    <t>function_app.py:1167:VECTOR_FIELD = os.environ["AZURE_SEARCH_VECTOR_FIELD"]</t>
+  </si>
+  <si>
+    <t>function_app.py:1168:SOURCE_FIELD = os.environ["AZURE_SEARCH_SOURCE_FIELD"]</t>
+  </si>
+  <si>
+    <t>function_app.py:1175:AZURE_OPENAI_ENDPOINT = os.environ["AZURE_OPENAI_ENDPOINT"]</t>
+  </si>
+  <si>
+    <t>function_app.py:1176:AZURE_OPENAI_DEPLOYMENT = os.environ["AZURE_OPENAI_DEPLOYMENT"]</t>
+  </si>
+  <si>
+    <t>function_app.py:1183:POLICY_SYSTEM_PROMPT_VERSION = os.environ[</t>
+  </si>
+  <si>
+    <t>function_app.py:1187:POLICY_SYSTEM_PROMPT_FILE = os.environ[</t>
+  </si>
+  <si>
+    <t>function_app.py:1196:COSMOS_ENDPOINT = os.environ["COSMOS_ENDPOINT"]</t>
+  </si>
+  <si>
+    <t>function_app.py:1197:COSMOS_DATABASE = os.environ["COSMOS_DATABASE"]</t>
+  </si>
+  <si>
+    <t>function_app.py:1199:COSMOS_CONVERSATIONS_CONTAINER = os.environ[</t>
+  </si>
+  <si>
+    <t>function_app.py:1203:COSMOS_MESSAGES_CONTAINER = os.environ[</t>
+  </si>
+  <si>
+    <t>function_app.py:1211:COSMOS_MEMORIES_CONTAINER = os.environ[</t>
+  </si>
+  <si>
+    <t>function_app.py:1220:ENTRA_TENANT_ID = os.environ["ENTRA_TENANT_ID"]</t>
+  </si>
+  <si>
+    <t>function_app.py:1221:ENTRA_API_CLIENT_ID = os.environ["ENTRA_API_CLIENT_ID"]</t>
+  </si>
+  <si>
+    <t>function_app.py:17579:                if os.getenv(name) is None</t>
+  </si>
+  <si>
+    <t>function_app.py:21452:    os.getenv("I14_DEV_VALIDATION_ENABLED", "false")</t>
+  </si>
+  <si>
+    <t>test_group_overage.py:17:    os.environ.setdefault(key, str(value))</t>
+  </si>
+  <si>
+    <t>test_step20.py:22:        os.environ.setdefault(key, str(value))</t>
+  </si>
+  <si>
+    <t>test_step21.py:17:        os.environ.setdefault(key, str(value))</t>
+  </si>
+  <si>
+    <t>test_step23.py:17:        os.environ.setdefault(key, str(value))</t>
+  </si>
+  <si>
+    <t>test_step29.py:145:    endpoint = os.getenv(</t>
+  </si>
+  <si>
+    <t>test_step29.py:150:    access_token = os.getenv(</t>
+  </si>
+  <si>
+    <t>validate_i29_step2.py:9:    os.environ[key] = str(value)</t>
+  </si>
+  <si>
+    <t>tests\conftest.py:42:    os.environ.setdefault(_name, _value)</t>
+  </si>
+  <si>
+    <t>tests\integration\conftest.py:66:        os.environ[name] = str(value)</t>
+  </si>
+  <si>
+    <t>tests\integration\conftest.py:69:    os.environ["LONG_TERM_MEMORY_ENABLED"] = "true"</t>
+  </si>
+  <si>
+    <t>tests\integration\conftest.py:81:    if os.getenv("RUN_COSMOS_INTEGRATION_TESTS", "").strip().lower() not in {</t>
   </si>
 </sst>
 </file>
@@ -628,7 +947,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -708,9 +1027,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -725,6 +1041,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -983,29 +1308,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G24"/>
+  <sheetPr>
+    <tabColor rgb="FFC00000"/>
+  </sheetPr>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="8" style="6" customWidth="1"/>
-    <col min="2" max="2" width="35.6640625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="38.73046875" style="4" customWidth="1"/>
     <col min="3" max="3" width="16" style="4" customWidth="1"/>
     <col min="4" max="4" width="34" style="4" customWidth="1"/>
     <col min="5" max="5" width="42" style="4" customWidth="1"/>
     <col min="6" max="6" width="55" style="4" customWidth="1"/>
-    <col min="7" max="7" width="18" style="28" customWidth="1"/>
+    <col min="7" max="7" width="18" style="27" customWidth="1"/>
     <col min="8" max="16384" width="9.06640625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="14" customHeight="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="2" spans="1:7" s="1" customFormat="1" ht="12" customHeight="1">
       <c r="A2" s="13" t="s">
@@ -1034,22 +1362,22 @@
       <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="29" t="s">
+      <c r="C3" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="29" t="s">
+      <c r="E3" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="30" t="s">
+      <c r="F3" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="29" t="s">
+      <c r="G3" s="28" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1057,22 +1385,22 @@
       <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="29" t="s">
+      <c r="C4" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="29" t="s">
+      <c r="E4" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="30" t="s">
+      <c r="F4" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="29" t="s">
+      <c r="G4" s="28" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1080,22 +1408,22 @@
       <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="29" t="s">
+      <c r="E5" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="29" t="s">
+      <c r="F5" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="29" t="s">
+      <c r="G5" s="28" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1103,22 +1431,22 @@
       <c r="A6" s="6">
         <v>4</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="29" t="s">
+      <c r="C6" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="31" t="s">
+      <c r="E6" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="29" t="s">
+      <c r="F6" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="G6" s="29" t="s">
+      <c r="G6" s="28" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1126,22 +1454,22 @@
       <c r="A7" s="6">
         <v>5</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="29" t="s">
+      <c r="C7" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="29" t="s">
+      <c r="E7" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="30" t="s">
+      <c r="F7" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="29" t="s">
+      <c r="G7" s="28" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1149,22 +1477,22 @@
       <c r="A8" s="6">
         <v>6</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="29" t="s">
+      <c r="C8" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="29" t="s">
+      <c r="E8" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="30" t="s">
+      <c r="F8" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="G8" s="29" t="s">
+      <c r="G8" s="28" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1172,22 +1500,22 @@
       <c r="A9" s="6">
         <v>7</v>
       </c>
-      <c r="B9" s="29" t="s">
+      <c r="B9" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="29" t="s">
+      <c r="C9" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="29" t="s">
+      <c r="E9" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="F9" s="29" t="s">
+      <c r="F9" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="G9" s="29" t="s">
+      <c r="G9" s="28" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1195,22 +1523,22 @@
       <c r="A10" s="6">
         <v>8</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="29" t="s">
+      <c r="C10" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="29" t="s">
+      <c r="E10" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="29" t="s">
+      <c r="F10" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="G10" s="29" t="s">
+      <c r="G10" s="28" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1218,242 +1546,530 @@
       <c r="A11" s="6">
         <v>9</v>
       </c>
-      <c r="B11" s="29" t="s">
+      <c r="B11" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="29" t="s">
+      <c r="C11" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="30" t="s">
+        <v>187</v>
+      </c>
+      <c r="E11" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="29" t="s">
+      <c r="F11" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="F11" s="29" t="s">
+      <c r="G11" s="28" t="s">
         <v>45</v>
-      </c>
-      <c r="G11" s="29" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:7" s="2" customFormat="1" ht="30" customHeight="1">
       <c r="A12" s="6">
         <v>10</v>
       </c>
-      <c r="B12" s="29" t="s">
+      <c r="B12" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="30" t="s">
+        <v>187</v>
+      </c>
+      <c r="E12" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="29" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" s="29" t="s">
+      <c r="F12" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="F12" s="29" t="s">
-        <v>49</v>
-      </c>
-      <c r="G12" s="29" t="s">
-        <v>46</v>
+      <c r="G12" s="28" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="2" customFormat="1" ht="30" customHeight="1">
       <c r="A13" s="6">
         <v>11</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="C13" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" s="29" t="s">
+      <c r="E13" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="E13" s="29" t="s">
+      <c r="F13" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="F13" s="29" t="s">
-        <v>53</v>
-      </c>
-      <c r="G13" s="29" t="s">
-        <v>46</v>
+      <c r="G13" s="28" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:7" s="2" customFormat="1" ht="30" customHeight="1">
       <c r="A14" s="6">
         <v>12</v>
       </c>
-      <c r="B14" s="29" t="s">
+      <c r="B14" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="C14" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="E14" s="29" t="s">
+      <c r="F14" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="F14" s="29" t="s">
-        <v>56</v>
-      </c>
-      <c r="G14" s="29" t="s">
-        <v>46</v>
+      <c r="G14" s="28" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="2" customFormat="1" ht="30" customHeight="1">
       <c r="A15" s="6">
         <v>13</v>
       </c>
-      <c r="B15" s="29" t="s">
+      <c r="B15" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="29" t="s">
+      <c r="E15" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="E15" s="29" t="s">
+      <c r="F15" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="F15" s="29" t="s">
-        <v>60</v>
-      </c>
-      <c r="G15" s="29" t="s">
-        <v>46</v>
+      <c r="G15" s="28" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:7" s="2" customFormat="1" ht="30" customHeight="1">
       <c r="A16" s="6">
         <v>14</v>
       </c>
-      <c r="B16" s="29" t="s">
+      <c r="B16" s="28" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="E16" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="C16" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="E16" s="29" t="s">
+      <c r="F16" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="F16" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="G16" s="29" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" s="2" customFormat="1">
+      <c r="G16" s="28" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="2" customFormat="1" ht="27" customHeight="1">
       <c r="A17" s="6"/>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="C17" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="G17" s="28"/>
+    </row>
+    <row r="18" spans="1:7" s="2" customFormat="1" ht="27" customHeight="1">
+      <c r="A18" s="6"/>
+      <c r="B18" s="28" t="s">
         <v>160</v>
       </c>
-      <c r="C17" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D17" s="29" t="s">
+      <c r="C18" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="F17" s="29" t="s">
-        <v>114</v>
-      </c>
-      <c r="G17" s="29"/>
-    </row>
-    <row r="18" spans="1:7" s="2" customFormat="1">
-      <c r="A18" s="6"/>
-      <c r="B18" s="2" t="s">
+      <c r="F18" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="G18" s="28"/>
+    </row>
+    <row r="19" spans="1:7" s="2" customFormat="1" ht="27" customHeight="1">
+      <c r="A19" s="6"/>
+      <c r="B19" s="28" t="s">
+        <v>164</v>
+      </c>
+      <c r="C19" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" s="28" t="s">
         <v>161</v>
       </c>
-      <c r="C18" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="29" t="s">
+      <c r="G19" s="28"/>
+    </row>
+    <row r="20" spans="1:7" s="2" customFormat="1" ht="27" customHeight="1">
+      <c r="A20" s="6"/>
+      <c r="B20" s="28" t="s">
+        <v>162</v>
+      </c>
+      <c r="C20" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="F18" s="29" t="s">
-        <v>117</v>
-      </c>
-      <c r="G18" s="29"/>
-    </row>
-    <row r="19" spans="1:7" s="2" customFormat="1">
-      <c r="A19" s="6"/>
-      <c r="B19" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="C19" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="F19" s="29" t="s">
+      <c r="F20" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20" s="28"/>
+    </row>
+    <row r="21" spans="1:7" s="2" customFormat="1" ht="27" customHeight="1">
+      <c r="A21" s="6"/>
+      <c r="B21" s="28" t="s">
         <v>163</v>
       </c>
-      <c r="G19" s="29"/>
-    </row>
-    <row r="20" spans="1:7" s="2" customFormat="1">
-      <c r="A20" s="6"/>
-      <c r="B20" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C20" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D20" s="29" t="s">
+      <c r="C21" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="F20" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="G20" s="29"/>
-    </row>
-    <row r="21" spans="1:7" s="2" customFormat="1" ht="28.5">
-      <c r="A21" s="6"/>
-      <c r="B21" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="C21" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D21" s="29" t="s">
+      <c r="F21" s="31" t="s">
+        <v>41</v>
+      </c>
+      <c r="G21" s="28"/>
+    </row>
+    <row r="22" spans="1:7" s="2" customFormat="1" ht="27" customHeight="1">
+      <c r="A22" s="6"/>
+      <c r="B22" s="28" t="s">
+        <v>92</v>
+      </c>
+      <c r="C22" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="F21" s="32" t="s">
-        <v>41</v>
-      </c>
-      <c r="G21" s="29"/>
-    </row>
-    <row r="22" spans="1:7" s="2" customFormat="1">
-      <c r="A22" s="6"/>
-      <c r="B22" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C22" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" s="29" t="s">
-        <v>15</v>
-      </c>
-      <c r="F22" s="32" t="s">
+      <c r="F22" s="31" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:7" s="2" customFormat="1">
       <c r="A23" s="6"/>
+      <c r="B23" s="28" t="s">
+        <v>165</v>
+      </c>
+      <c r="C23" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" s="30"/>
+      <c r="F23" s="31" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="24" spans="1:7" s="2" customFormat="1">
       <c r="A24" s="6"/>
+      <c r="B24" s="28" t="s">
+        <v>166</v>
+      </c>
+      <c r="C24" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="E24" s="30"/>
+      <c r="F24" s="28" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="B25" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="C25" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="E25" s="30"/>
+      <c r="F25" s="28" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="B26" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="C26" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="E26" s="30"/>
+      <c r="F26" s="28" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="B27" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="C27" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="E27" s="30"/>
+      <c r="F27" s="28" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="B28" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="C28" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="E28" s="30"/>
+      <c r="F28" s="28" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="B29" s="28" t="s">
+        <v>170</v>
+      </c>
+      <c r="C29" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="30" t="s">
+        <v>187</v>
+      </c>
+      <c r="E29" s="30"/>
+      <c r="F29" s="31" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="B30" s="28" t="s">
+        <v>171</v>
+      </c>
+      <c r="C30" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="30" t="s">
+        <v>187</v>
+      </c>
+      <c r="E30" s="30"/>
+      <c r="F30" s="28" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="B31" s="28" t="s">
+        <v>172</v>
+      </c>
+      <c r="C31" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" s="30" t="s">
+        <v>187</v>
+      </c>
+      <c r="E31" s="30"/>
+      <c r="F31" s="30" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="B32" s="28" t="s">
+        <v>173</v>
+      </c>
+      <c r="C32" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32" s="30" t="s">
+        <v>187</v>
+      </c>
+      <c r="E32" s="30"/>
+      <c r="F32" s="30" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6">
+      <c r="B33" s="28" t="s">
+        <v>174</v>
+      </c>
+      <c r="C33" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33" s="30" t="s">
+        <v>187</v>
+      </c>
+      <c r="E33" s="30"/>
+      <c r="F33" s="30" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6">
+      <c r="B34" s="28" t="s">
+        <v>175</v>
+      </c>
+      <c r="C34" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" s="30" t="s">
+        <v>188</v>
+      </c>
+      <c r="F34" s="31" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6">
+      <c r="B35" s="28" t="s">
+        <v>176</v>
+      </c>
+      <c r="C35" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D35" s="30" t="s">
+        <v>188</v>
+      </c>
+      <c r="F35" s="30" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6">
+      <c r="B36" s="28" t="s">
+        <v>177</v>
+      </c>
+      <c r="C36" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D36" s="30" t="s">
+        <v>189</v>
+      </c>
+      <c r="F36" s="30" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6">
+      <c r="B37" s="28" t="s">
+        <v>178</v>
+      </c>
+      <c r="C37" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D37" s="30" t="s">
+        <v>189</v>
+      </c>
+      <c r="F37" s="30" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6">
+      <c r="B38" s="28" t="s">
+        <v>179</v>
+      </c>
+      <c r="C38" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D38" s="30" t="s">
+        <v>191</v>
+      </c>
+      <c r="F38" s="30" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6">
+      <c r="B39" s="28" t="s">
+        <v>180</v>
+      </c>
+      <c r="C39" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D39" s="30" t="s">
+        <v>191</v>
+      </c>
+      <c r="F39" s="30" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6">
+      <c r="B40" s="28" t="s">
+        <v>181</v>
+      </c>
+      <c r="C40" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D40" s="30" t="s">
+        <v>191</v>
+      </c>
+      <c r="F40" s="30" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6">
+      <c r="B41" s="28" t="s">
+        <v>182</v>
+      </c>
+      <c r="C41" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D41" s="30" t="s">
+        <v>195</v>
+      </c>
+      <c r="F41" s="32" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6">
+      <c r="B42" s="28" t="s">
+        <v>183</v>
+      </c>
+      <c r="C42" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D42" s="30" t="s">
+        <v>195</v>
+      </c>
+      <c r="F42" s="30" t="s">
+        <v>194</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:G42" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
@@ -1475,6 +2091,9 @@
     <hyperlink ref="F20" r:id="rId5" xr:uid="{43A3D446-E6D1-4BAB-83D6-CA00B2AD4B1C}"/>
     <hyperlink ref="F21" r:id="rId6" xr:uid="{CC5D8445-06EA-49DE-98E7-C9E2A380AA4D}"/>
     <hyperlink ref="F22" r:id="rId7" xr:uid="{6585A9C8-FB75-4280-BFDD-F1E3AC60A7B9}"/>
+    <hyperlink ref="F23" r:id="rId8" xr:uid="{D4D39A54-2E11-4AAC-9782-F5EB1D6DA592}"/>
+    <hyperlink ref="F29" r:id="rId9" xr:uid="{5D30BC6B-80BE-42A1-BC84-B8EA5643F1D5}"/>
+    <hyperlink ref="F34" r:id="rId10" xr:uid="{AB03932A-0EF1-4511-8992-991F60C206A0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1482,31 +2101,34 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr>
+    <tabColor rgb="FF7030A0"/>
+  </sheetPr>
   <dimension ref="A1:F134"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="31" style="4" customWidth="1"/>
     <col min="2" max="2" width="42" style="4" customWidth="1"/>
     <col min="3" max="3" width="20" style="6" customWidth="1"/>
-    <col min="4" max="4" width="58" style="4" customWidth="1"/>
+    <col min="4" max="4" width="61.6640625" style="4" customWidth="1"/>
     <col min="5" max="5" width="18" style="6" customWidth="1"/>
     <col min="6" max="6" width="46" customWidth="1"/>
     <col min="7" max="16384" width="9.06640625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="14" customHeight="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="33" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+    </row>
+    <row r="2" spans="1:6" ht="19.899999999999999" customHeight="1">
+      <c r="A2" s="18" t="s">
         <v>64</v>
-      </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-    </row>
-    <row r="2" spans="1:6" ht="12" customHeight="1">
-      <c r="A2" s="18" t="s">
-        <v>65</v>
       </c>
       <c r="B2" s="18" t="s">
         <v>4</v>
@@ -1515,18 +2137,18 @@
         <v>3</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E2" s="18" t="s">
         <v>7</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A3" s="19" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B3" s="19" t="s">
         <v>15</v>
@@ -1546,7 +2168,7 @@
     </row>
     <row r="4" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A4" s="22" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B4" s="22" t="s">
         <v>19</v>
@@ -1561,15 +2183,15 @@
         <v>13</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A5" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5" s="22" t="s">
         <v>71</v>
-      </c>
-      <c r="B5" s="22" t="s">
-        <v>72</v>
       </c>
       <c r="C5" s="23" t="s">
         <v>9</v>
@@ -1581,115 +2203,115 @@
         <v>13</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:6" s="2" customFormat="1" ht="26.1" customHeight="1">
       <c r="A6" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C6" s="20" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E6" s="25" t="s">
         <v>13</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A7" s="22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C7" s="23" t="s">
         <v>18</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E7" s="25" t="s">
         <v>13</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:6" s="2" customFormat="1" ht="24.6" customHeight="1">
       <c r="A8" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="C8" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="D8" s="24" t="s">
         <v>81</v>
-      </c>
-      <c r="D8" s="24" t="s">
-        <v>82</v>
       </c>
       <c r="E8" s="25" t="s">
         <v>13</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="2" customFormat="1" ht="30.95" customHeight="1">
       <c r="A9" s="22" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="D9" s="25" t="s">
         <v>84</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>80</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="D9" s="25" t="s">
-        <v>85</v>
       </c>
       <c r="E9" s="25" t="s">
         <v>13</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A10" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="24" t="s">
         <v>87</v>
-      </c>
-      <c r="B10" s="22" t="s">
-        <v>80</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="D10" s="24" t="s">
-        <v>88</v>
       </c>
       <c r="E10" s="25" t="s">
         <v>13</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A11" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="B11" s="22" t="s">
         <v>90</v>
-      </c>
-      <c r="B11" s="22" t="s">
-        <v>91</v>
       </c>
       <c r="C11" s="23" t="s">
         <v>9</v>
@@ -1701,15 +2323,15 @@
         <v>13</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A12" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" s="22" t="s">
         <v>93</v>
-      </c>
-      <c r="B12" s="22" t="s">
-        <v>94</v>
       </c>
       <c r="C12" s="23" t="s">
         <v>9</v>
@@ -1721,32 +2343,32 @@
         <v>13</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A13" s="22" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C13" s="23" t="s">
         <v>18</v>
       </c>
       <c r="D13" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E13" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" s="17" t="s">
         <v>97</v>
-      </c>
-      <c r="E13" s="25" t="s">
-        <v>46</v>
-      </c>
-      <c r="F13" s="17" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A14" s="22" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B14" s="22" t="s">
         <v>28</v>
@@ -1755,7 +2377,7 @@
         <v>9</v>
       </c>
       <c r="D14" s="24" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E14" s="25" t="s">
         <v>13</v>
@@ -1766,27 +2388,27 @@
     </row>
     <row r="15" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A15" s="22" t="s">
+        <v>100</v>
+      </c>
+      <c r="B15" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="C15" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="24" t="s">
         <v>102</v>
-      </c>
-      <c r="C15" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="24" t="s">
-        <v>103</v>
       </c>
       <c r="E15" s="25" t="s">
         <v>13</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A16" s="22" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B16" s="22" t="s">
         <v>28</v>
@@ -1795,18 +2417,18 @@
         <v>9</v>
       </c>
       <c r="D16" s="24" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E16" s="25" t="s">
         <v>13</v>
       </c>
       <c r="F16" s="17" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="17" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A17" s="22" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B17" s="22" t="s">
         <v>28</v>
@@ -1814,19 +2436,19 @@
       <c r="C17" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="D17" s="24" t="s">
-        <v>109</v>
+      <c r="D17" s="34" t="s">
+        <v>108</v>
       </c>
       <c r="E17" s="25" t="s">
         <v>13</v>
       </c>
       <c r="F17" s="17" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A18" s="22" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B18" s="22" t="s">
         <v>28</v>
@@ -1841,12 +2463,12 @@
         <v>13</v>
       </c>
       <c r="F18" s="17" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="19" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A19" s="22" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B19" s="22" t="s">
         <v>15</v>
@@ -1855,38 +2477,38 @@
         <v>9</v>
       </c>
       <c r="D19" s="24" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E19" s="25" t="s">
         <v>13</v>
       </c>
       <c r="F19" s="17" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A20" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="C20" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="24" t="s">
         <v>116</v>
-      </c>
-      <c r="B20" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="C20" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="D20" s="24" t="s">
-        <v>117</v>
       </c>
       <c r="E20" s="25" t="s">
         <v>13</v>
       </c>
       <c r="F20" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A21" s="22" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B21" s="22" t="s">
         <v>15</v>
@@ -1895,201 +2517,201 @@
         <v>9</v>
       </c>
       <c r="D21" s="24" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E21" s="25" t="s">
         <v>13</v>
       </c>
       <c r="F21" s="17" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="22" spans="1:6" s="2" customFormat="1" ht="18.95" customHeight="1">
       <c r="A22" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="B22" s="22" t="s">
         <v>122</v>
       </c>
-      <c r="B22" s="22" t="s">
+      <c r="C22" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="F22" s="17" t="s">
         <v>123</v>
-      </c>
-      <c r="C22" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="E22" s="25" t="s">
-        <v>46</v>
-      </c>
-      <c r="F22" s="17" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="23" spans="1:6" s="2" customFormat="1" ht="24.75" customHeight="1">
       <c r="A23" s="22" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B23" s="22" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C23" s="23" t="s">
         <v>9</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E23" s="25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F23" s="17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="24" spans="1:6" s="2" customFormat="1" ht="23.65" customHeight="1">
       <c r="A24" s="22" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B24" s="22" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C24" s="23" t="s">
         <v>9</v>
       </c>
       <c r="D24" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E24" s="25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F24" s="17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="25" spans="1:6" s="2" customFormat="1" ht="19.149999999999999" customHeight="1">
       <c r="A25" s="22" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B25" s="22" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C25" s="23" t="s">
         <v>9</v>
       </c>
       <c r="D25" s="26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E25" s="25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F25" s="17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="26" spans="1:6" s="2" customFormat="1" ht="19.149999999999999" customHeight="1">
       <c r="A26" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="B26" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="B26" s="22" t="s">
-        <v>129</v>
-      </c>
       <c r="C26" s="23" t="s">
         <v>9</v>
       </c>
       <c r="D26" s="25" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E26" s="25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F26" s="17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="27" spans="1:6" s="2" customFormat="1" ht="19.149999999999999" customHeight="1">
       <c r="A27" s="22" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B27" s="22" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C27" s="23" t="s">
         <v>9</v>
       </c>
       <c r="D27" s="25" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E27" s="25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F27" s="17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="28" spans="1:6" s="2" customFormat="1" ht="19.149999999999999" customHeight="1">
       <c r="A28" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B28" s="22" t="s">
+        <v>128</v>
+      </c>
+      <c r="C28" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" s="25" t="s">
         <v>131</v>
       </c>
-      <c r="B28" s="22" t="s">
-        <v>129</v>
-      </c>
-      <c r="C28" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="D28" s="25" t="s">
-        <v>132</v>
-      </c>
       <c r="E28" s="25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F28" s="17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="29" spans="1:6" s="2" customFormat="1" ht="19.149999999999999" customHeight="1">
       <c r="A29" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="B29" s="22" t="s">
+        <v>128</v>
+      </c>
+      <c r="C29" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="26" t="s">
         <v>133</v>
       </c>
-      <c r="B29" s="22" t="s">
-        <v>129</v>
-      </c>
-      <c r="C29" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="D29" s="26" t="s">
-        <v>134</v>
-      </c>
       <c r="E29" s="25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F29" s="17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="30" spans="1:6" s="2" customFormat="1" ht="19.149999999999999" customHeight="1">
       <c r="A30" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="B30" s="22" t="s">
+        <v>128</v>
+      </c>
+      <c r="C30" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="25" t="s">
         <v>135</v>
       </c>
-      <c r="B30" s="22" t="s">
-        <v>129</v>
-      </c>
-      <c r="C30" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="D30" s="25" t="s">
-        <v>136</v>
-      </c>
       <c r="E30" s="25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F30" s="17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="31" spans="1:6" s="2" customFormat="1" ht="19.149999999999999" customHeight="1">
       <c r="A31" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="B31" s="22" t="s">
         <v>137</v>
-      </c>
-      <c r="B31" s="22" t="s">
-        <v>138</v>
       </c>
       <c r="C31" s="23" t="s">
         <v>9</v>
@@ -2098,18 +2720,18 @@
         <v>17</v>
       </c>
       <c r="E31" s="25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F31" s="17" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="32" spans="1:6" s="2" customFormat="1" ht="19.149999999999999" customHeight="1">
       <c r="A32" s="19" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B32" s="22" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C32" s="20" t="s">
         <v>9</v>
@@ -2118,90 +2740,90 @@
         <v>21</v>
       </c>
       <c r="E32" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F32" s="17" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33" spans="1:6" s="2" customFormat="1" ht="19.149999999999999" customHeight="1">
       <c r="A33" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="B33" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="B33" s="22" t="s">
+      <c r="C33" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="C33" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="D33" s="16" t="s">
+      <c r="E33" s="17" t="s">
         <v>144</v>
       </c>
-      <c r="E33" s="17" t="s">
+      <c r="F33" s="17" t="s">
         <v>145</v>
-      </c>
-      <c r="F33" s="17" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="34" spans="1:6" s="2" customFormat="1" ht="19.149999999999999" customHeight="1">
       <c r="A34" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="B34" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="B34" s="22" t="s">
+      <c r="C34" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="C34" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="D34" s="16" t="s">
+      <c r="E34" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="F34" s="17" t="s">
         <v>149</v>
-      </c>
-      <c r="E34" s="17" t="s">
-        <v>145</v>
-      </c>
-      <c r="F34" s="17" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="35" spans="1:6" s="2" customFormat="1" ht="19.149999999999999" customHeight="1">
       <c r="A35" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="B35" s="22" t="s">
         <v>151</v>
       </c>
-      <c r="B35" s="22" t="s">
+      <c r="C35" s="23" t="s">
         <v>152</v>
       </c>
-      <c r="C35" s="23" t="s">
+      <c r="D35" s="26" t="s">
         <v>153</v>
-      </c>
-      <c r="D35" s="26" t="s">
-        <v>154</v>
       </c>
       <c r="E35" s="25" t="s">
         <v>26</v>
       </c>
       <c r="F35" s="17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="36" spans="1:6" s="2" customFormat="1" ht="19.149999999999999" customHeight="1">
       <c r="A36" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="B36" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="B36" s="22" t="s">
+      <c r="C36" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="C36" s="23" t="s">
-        <v>158</v>
-      </c>
       <c r="D36" s="26" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E36" s="25" t="s">
         <v>26</v>
       </c>
       <c r="F36" s="17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="37" spans="1:6" s="2" customFormat="1" ht="19.149999999999999" customHeight="1">
@@ -2567,7 +3189,401 @@
     <hyperlink ref="D48" r:id="rId8" display="https://policy-assist-orchestration-func-app-dev-cxarefhbeef6e6d7.westus3-01.azurewebsites.net/api/policy-chat" xr:uid="{00000000-0004-0000-0100-000007000000}"/>
     <hyperlink ref="D49" r:id="rId9" display="https://polite-ground-0d2a97a1e.6.azurestaticapps.net/" xr:uid="{00000000-0004-0000-0100-000008000000}"/>
     <hyperlink ref="D50" r:id="rId10" display="http://localhost:5173/" xr:uid="{00000000-0004-0000-0100-000009000000}"/>
+    <hyperlink ref="D17" r:id="rId11" xr:uid="{9BD680F8-27A1-4C8B-8469-D18F3E50EE44}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF156733-0289-49EA-8EC5-94A20D685CBE}">
+  <sheetPr>
+    <tabColor theme="8" tint="-0.249977111117893"/>
+  </sheetPr>
+  <dimension ref="A2:A76"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="91.59765625" customWidth="1"/>
+    <col min="2" max="2" width="59.73046875" customWidth="1"/>
+    <col min="3" max="3" width="28.86328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1">
+      <c r="A41" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1">
+      <c r="A64" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1">
+      <c r="A67" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1">
+      <c r="A69" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1">
+      <c r="A71" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1">
+      <c r="A73" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1">
+      <c r="A74" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76" t="s">
+        <v>270</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>